<commit_message>
Document tower balance updates and expand validation coverage
</commit_message>
<xml_diff>
--- a/outputs/01a073f8-7757-7fd0-acb0-5b552511c00b/Enemy_and_Tower_Stats.xlsx
+++ b/outputs/01a073f8-7757-7fd0-acb0-5b552511c00b/Enemy_and_Tower_Stats.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Towers" sheetId="1" r:id="R09ff55954b7247f5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Enemies" sheetId="2" r:id="R2b505b793f424de2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Towers" sheetId="1" r:id="R5efc085267bb49f5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Enemies" sheetId="2" r:id="Rd8ea0b4229af40d7"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -83,8 +83,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="TowersStats" displayName="TowersStats" ref="A7:G16" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A7:G16"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="TowersStats" displayName="TowersStats" ref="A7:G19" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A7:G19"/>
   <x:tableColumns count="7">
     <x:tableColumn id="1" name="Tower"/>
     <x:tableColumn id="2" name="Level"/>
@@ -503,16 +503,16 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="C12" s="7" t="n">
-        <x:v>25</x:v>
+        <x:v>24</x:v>
       </x:c>
       <x:c r="D12" s="7" t="n">
-        <x:v>1.25</x:v>
+        <x:v>1.3</x:v>
       </x:c>
       <x:c r="E12" s="7" t="n">
         <x:v>140</x:v>
       </x:c>
       <x:c r="F12" s="7" t="n">
-        <x:v>58</x:v>
+        <x:v>56</x:v>
       </x:c>
       <x:c r="G12" s="7" t="n">
         <x:v>120</x:v>
@@ -526,16 +526,16 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="C13" s="7" t="n">
-        <x:v>45</x:v>
+        <x:v>36</x:v>
       </x:c>
       <x:c r="D13" s="7" t="n">
-        <x:v>1</x:v>
+        <x:v>1.1</x:v>
       </x:c>
       <x:c r="E13" s="7" t="n">
         <x:v>154</x:v>
       </x:c>
       <x:c r="F13" s="7" t="n">
-        <x:v>70</x:v>
+        <x:v>66</x:v>
       </x:c>
       <x:c r="G13" s="7" t="n">
         <x:v>200</x:v>
@@ -575,7 +575,7 @@
         <x:v>60</x:v>
       </x:c>
       <x:c r="D15" s="7" t="n">
-        <x:v>1.5</x:v>
+        <x:v>1.35</x:v>
       </x:c>
       <x:c r="E15" s="7" t="n">
         <x:v>173</x:v>
@@ -598,7 +598,7 @@
         <x:v>90</x:v>
       </x:c>
       <x:c r="D16" s="7" t="n">
-        <x:v>1.2</x:v>
+        <x:v>0.9</x:v>
       </x:c>
       <x:c r="E16" s="7" t="n">
         <x:v>189</x:v>
@@ -608,12 +608,81 @@
       </x:c>
       <x:c r="G16" s="7" t="n">
         <x:v>220</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17">
+      <x:c r="A17" t="str">
+        <x:v>Stormspire</x:v>
+      </x:c>
+      <x:c r="B17" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C17" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="D17" t="n">
+        <x:v>0.4</x:v>
+      </x:c>
+      <x:c r="E17" t="n">
+        <x:v>145</x:v>
+      </x:c>
+      <x:c r="F17" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G17" t="n">
+        <x:v>140</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18">
+      <x:c r="A18" t="str">
+        <x:v>Stormspire</x:v>
+      </x:c>
+      <x:c r="B18" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C18" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="D18" t="n">
+        <x:v>0.35</x:v>
+      </x:c>
+      <x:c r="E18" t="n">
+        <x:v>159</x:v>
+      </x:c>
+      <x:c r="F18" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G18" t="n">
+        <x:v>120</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19">
+      <x:c r="A19" t="str">
+        <x:v>Stormspire</x:v>
+      </x:c>
+      <x:c r="B19" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="C19" t="n">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="D19" t="n">
+        <x:v>0.3</x:v>
+      </x:c>
+      <x:c r="E19" t="n">
+        <x:v>173</x:v>
+      </x:c>
+      <x:c r="F19" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G19" t="n">
+        <x:v>200</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Radeb4bb52cdb4674"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra2310f470a0f4f81"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -703,7 +772,7 @@
         <x:v>Hollow</x:v>
       </x:c>
       <x:c r="B8" s="7" t="n">
-        <x:v>15</x:v>
+        <x:v>45</x:v>
       </x:c>
       <x:c r="C8" s="7" t="n">
         <x:v>0</x:v>
@@ -720,7 +789,7 @@
         <x:v>Wraith</x:v>
       </x:c>
       <x:c r="B9" s="7" t="n">
-        <x:v>12</x:v>
+        <x:v>36</x:v>
       </x:c>
       <x:c r="C9" s="7" t="n">
         <x:v>0</x:v>
@@ -737,7 +806,7 @@
         <x:v>Revenant</x:v>
       </x:c>
       <x:c r="B10" s="7" t="n">
-        <x:v>85</x:v>
+        <x:v>340</x:v>
       </x:c>
       <x:c r="C10" s="7" t="n">
         <x:v>0</x:v>
@@ -752,7 +821,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf281c01b3425434d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5d614008df8741b8"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Add level-four tower specializations and update balance references
</commit_message>
<xml_diff>
--- a/outputs/01a073f8-7757-7fd0-acb0-5b552511c00b/Enemy_and_Tower_Stats.xlsx
+++ b/outputs/01a073f8-7757-7fd0-acb0-5b552511c00b/Enemy_and_Tower_Stats.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Towers" sheetId="1" r:id="R5efc085267bb49f5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Enemies" sheetId="2" r:id="Rd8ea0b4229af40d7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Towers" sheetId="1" r:id="Rd4d84ed6712c4cfb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Enemies" sheetId="2" r:id="Rd50f38b21db84a11"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -14,10 +14,12 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:numFmts count="1">
+  <x:numFmts count="3">
     <x:numFmt numFmtId="200" formatCode="0.##"/>
+    <x:numFmt numFmtId="201" formatCode="0"/>
+    <x:numFmt numFmtId="202" formatCode="0.00"/>
   </x:numFmts>
-  <x:fonts count="5">
+  <x:fonts count="7">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -44,8 +46,19 @@
       <x:color rgb="FFFFFFFF"/>
       <x:name val="Arial"/>
     </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="12"/>
+      <x:color rgb="FF334155"/>
+      <x:name val="Carlito"/>
+    </x:font>
+    <x:font>
+      <x:sz val="11"/>
+      <x:color rgb="FF334155"/>
+      <x:name val="Arial"/>
+    </x:font>
   </x:fonts>
-  <x:fills count="3">
+  <x:fills count="5">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -57,6 +70,16 @@
         <x:fgColor rgb="FF334155"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFEAF3F8"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFFFFF"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
   <x:borders count="1">
     <x:border/>
@@ -64,7 +87,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="8">
+  <x:cellXfs count="20">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -75,6 +98,32 @@
       <x:alignment wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="200" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="202" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="6" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="6" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="6" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="6" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -83,8 +132,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="TowersStats" displayName="TowersStats" ref="A7:G19" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A7:G19"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="TowersStats" displayName="TowersStats" ref="A7:G27" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A7:G27"/>
   <x:tableColumns count="7">
     <x:tableColumn id="1" name="Tower"/>
     <x:tableColumn id="2" name="Level"/>
@@ -340,7 +389,7 @@
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="3" t="str">
-        <x:v>Source: balance.gd, TOWERS and TOWER_UPGRADES; combat.gd, tick and hit.</x:v>
+        <x:v>Source: balance.gd, TOWERS, TOWER_UPGRADES and BRANCHES; combat.gd, branch effects.</x:v>
       </x:c>
       <x:c r="B3" s="3"/>
       <x:c r="C3" s="3"/>
@@ -362,7 +411,7 @@
     </x:row>
     <x:row r="5">
       <x:c r="A5" s="3" t="str">
-        <x:v>To expand: press Tab in the last table cell to add a row. Use one row per tower level.</x:v>
+        <x:v>Level 4 is one permanent branch choice. Branch damage below excludes conditional bonuses; see effect rules below.</x:v>
       </x:c>
       <x:c r="B5" s="3"/>
       <x:c r="C5" s="3"/>
@@ -679,10 +728,319 @@
         <x:v>200</x:v>
       </x:c>
     </x:row>
+    <x:row r="20" ht="34" customHeight="1">
+      <x:c r="A20" s="8" t="str">
+        <x:v>Frostneedle</x:v>
+      </x:c>
+      <x:c r="B20" s="9" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="C20" s="9" t="n">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="D20" s="10" t="n">
+        <x:v>0.3</x:v>
+      </x:c>
+      <x:c r="E20" s="9" t="n">
+        <x:v>160</x:v>
+      </x:c>
+      <x:c r="F20" s="9" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G20" s="9" t="n">
+        <x:v>180</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="21" ht="34" customHeight="1">
+      <x:c r="A21" s="8" t="str">
+        <x:v>Thorn Volley</x:v>
+      </x:c>
+      <x:c r="B21" s="9" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="C21" s="9" t="n">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="D21" s="10" t="n">
+        <x:v>0.3</x:v>
+      </x:c>
+      <x:c r="E21" s="9" t="n">
+        <x:v>160</x:v>
+      </x:c>
+      <x:c r="F21" s="9" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G21" s="9" t="n">
+        <x:v>180</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="22" ht="34" customHeight="1">
+      <x:c r="A22" s="8" t="str">
+        <x:v>Cinderfield</x:v>
+      </x:c>
+      <x:c r="B22" s="9" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="C22" s="9" t="n">
+        <x:v>27</x:v>
+      </x:c>
+      <x:c r="D22" s="10" t="n">
+        <x:v>1.1</x:v>
+      </x:c>
+      <x:c r="E22" s="9" t="n">
+        <x:v>154</x:v>
+      </x:c>
+      <x:c r="F22" s="9" t="n">
+        <x:v>66</x:v>
+      </x:c>
+      <x:c r="G22" s="9" t="n">
+        <x:v>320</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="23" ht="34" customHeight="1">
+      <x:c r="A23" s="8" t="str">
+        <x:v>Rupture Pyre</x:v>
+      </x:c>
+      <x:c r="B23" s="9" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="C23" s="9" t="n">
+        <x:v>54</x:v>
+      </x:c>
+      <x:c r="D23" s="10" t="n">
+        <x:v>1.5</x:v>
+      </x:c>
+      <x:c r="E23" s="9" t="n">
+        <x:v>154</x:v>
+      </x:c>
+      <x:c r="F23" s="9" t="n">
+        <x:v>66</x:v>
+      </x:c>
+      <x:c r="G23" s="9" t="n">
+        <x:v>320</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="24" ht="34" customHeight="1">
+      <x:c r="A24" s="8" t="str">
+        <x:v>Grave Echo</x:v>
+      </x:c>
+      <x:c r="B24" s="9" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="C24" s="9" t="n">
+        <x:v>110</x:v>
+      </x:c>
+      <x:c r="D24" s="10" t="n">
+        <x:v>0.9</x:v>
+      </x:c>
+      <x:c r="E24" s="9" t="n">
+        <x:v>189</x:v>
+      </x:c>
+      <x:c r="F24" s="9" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G24" s="9" t="n">
+        <x:v>360</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="25" ht="34" customHeight="1">
+      <x:c r="A25" s="8" t="str">
+        <x:v>Doomstone</x:v>
+      </x:c>
+      <x:c r="B25" s="9" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="C25" s="9" t="n">
+        <x:v>90</x:v>
+      </x:c>
+      <x:c r="D25" s="10" t="n">
+        <x:v>0.9</x:v>
+      </x:c>
+      <x:c r="E25" s="9" t="n">
+        <x:v>189</x:v>
+      </x:c>
+      <x:c r="F25" s="9" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G25" s="9" t="n">
+        <x:v>360</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="26" ht="34" customHeight="1">
+      <x:c r="A26" s="8" t="str">
+        <x:v>Tempest Web</x:v>
+      </x:c>
+      <x:c r="B26" s="9" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="C26" s="9" t="n">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="D26" s="10" t="n">
+        <x:v>0.3</x:v>
+      </x:c>
+      <x:c r="E26" s="9" t="n">
+        <x:v>173</x:v>
+      </x:c>
+      <x:c r="F26" s="9" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G26" s="9" t="n">
+        <x:v>300</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="27" ht="34" customHeight="1">
+      <x:c r="A27" s="8" t="str">
+        <x:v>Thunderseal</x:v>
+      </x:c>
+      <x:c r="B27" s="9" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="C27" s="9" t="n">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="D27" s="10" t="n">
+        <x:v>0.3</x:v>
+      </x:c>
+      <x:c r="E27" s="9" t="n">
+        <x:v>173</x:v>
+      </x:c>
+      <x:c r="F27" s="9" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G27" s="9" t="n">
+        <x:v>300</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="29">
+      <x:c r="A29" s="11" t="str">
+        <x:v>Level 4 effect rules</x:v>
+      </x:c>
+      <x:c r="B29" s="11"/>
+      <x:c r="C29" s="11"/>
+      <x:c r="D29" s="11"/>
+      <x:c r="E29" s="11"/>
+      <x:c r="F29" s="11"/>
+      <x:c r="G29" s="11"/>
+    </x:row>
+    <x:row r="30" ht="55" customHeight="1">
+      <x:c r="A30" s="15" t="str">
+        <x:v>Frostneedle</x:v>
+      </x:c>
+      <x:c r="B30" s="15" t="str">
+        <x:v>Ashneedle branch. Hits slow movement 25% for 2 seconds. Further hits refresh duration, never stack the reduction. Icy blue body and crystal crown.</x:v>
+      </x:c>
+      <x:c r="C30" s="15"/>
+      <x:c r="D30" s="15"/>
+      <x:c r="E30" s="15"/>
+      <x:c r="F30" s="15"/>
+      <x:c r="G30" s="15"/>
+    </x:row>
+    <x:row r="31" ht="55" customHeight="1">
+      <x:c r="A31" s="19" t="str">
+        <x:v>Thorn Volley</x:v>
+      </x:c>
+      <x:c r="B31" s="19" t="str">
+        <x:v>Ashneedle branch. Five 15-damage arrows: center tracks the target; outer angles are -27.5°, -13.8°, +13.8°, +27.5°. Outer arrows travel straight, can miss, and hit the first enemy encountered. Five-pronged green launcher.</x:v>
+      </x:c>
+      <x:c r="C31" s="19"/>
+      <x:c r="D31" s="19"/>
+      <x:c r="E31" s="19"/>
+      <x:c r="F31" s="19"/>
+      <x:c r="G31" s="19"/>
+    </x:row>
+    <x:row r="32" ht="55" customHeight="1">
+      <x:c r="A32" s="15" t="str">
+        <x:v>Cinderfield</x:v>
+      </x:c>
+      <x:c r="B32" s="15" t="str">
+        <x:v>Pyre branch. Each 27-damage blast leaves fire for 3 seconds at 12 damage per second. Overlapping patches from the same tower refresh and cannot stack damage on an enemy. Cracked ember basin and glowing scorch marks.</x:v>
+      </x:c>
+      <x:c r="C32" s="15"/>
+      <x:c r="D32" s="15"/>
+      <x:c r="E32" s="15"/>
+      <x:c r="F32" s="15"/>
+      <x:c r="G32" s="15"/>
+    </x:row>
+    <x:row r="33" ht="55" customHeight="1">
+      <x:c r="A33" s="19" t="str">
+        <x:v>Rupture Pyre</x:v>
+      </x:c>
+      <x:c r="B33" s="19" t="str">
+        <x:v>Pyre branch. 54 damage every 1.5 seconds. Pushes enemies backward 20 units along their road, or 5 units for Revenants. Push immunity lasts 1 second. Reinforced brazier and orange shockwaves.</x:v>
+      </x:c>
+      <x:c r="C33" s="19"/>
+      <x:c r="D33" s="19"/>
+      <x:c r="E33" s="19"/>
+      <x:c r="F33" s="19"/>
+      <x:c r="G33" s="19"/>
+    </x:row>
+    <x:row r="34" ht="55" customHeight="1">
+      <x:c r="A34" s="15" t="str">
+        <x:v>Grave Echo</x:v>
+      </x:c>
+      <x:c r="B34" s="15" t="str">
+        <x:v>Obelisk branch. 110-damage orb creates up to five seeking fragments at 22 damage each. Distinct enemies within 90 units of impact; excludes the original target. Unused fragments fade. Fractured violet crystal and curved shard trails.</x:v>
+      </x:c>
+      <x:c r="C34" s="15"/>
+      <x:c r="D34" s="15"/>
+      <x:c r="E34" s="15"/>
+      <x:c r="F34" s="15"/>
+      <x:c r="G34" s="15"/>
+    </x:row>
+    <x:row r="35" ht="55" customHeight="1">
+      <x:c r="A35" s="19" t="str">
+        <x:v>Doomstone</x:v>
+      </x:c>
+      <x:c r="B35" s="19" t="str">
+        <x:v>Obelisk branch. First hit deals 90. Consecutive hits add 20% of base damage per stack, capped at five stacks and 180 damage. Switching targets resets this tower’s buildup. Dark floating monolith and brightening curse symbols.</x:v>
+      </x:c>
+      <x:c r="C35" s="19"/>
+      <x:c r="D35" s="19"/>
+      <x:c r="E35" s="19"/>
+      <x:c r="F35" s="19"/>
+      <x:c r="G35" s="19"/>
+    </x:row>
+    <x:row r="36" ht="55" customHeight="1">
+      <x:c r="A36" s="15" t="str">
+        <x:v>Tempest Web</x:v>
+      </x:c>
+      <x:c r="B36" s="15" t="str">
+        <x:v>Stormspire branch. Up to five primary hits at 7 damage. Each can arc within 60 units to one distinct additional enemy for 3.5 damage; primary targets are excluded from arcs. Arcs can exceed 173-unit tower range. Branching metal crown.</x:v>
+      </x:c>
+      <x:c r="C36" s="15"/>
+      <x:c r="D36" s="15"/>
+      <x:c r="E36" s="15"/>
+      <x:c r="F36" s="15"/>
+      <x:c r="G36" s="15"/>
+    </x:row>
+    <x:row r="37" ht="55" customHeight="1">
+      <x:c r="A37" s="19" t="str">
+        <x:v>Thunderseal</x:v>
+      </x:c>
+      <x:c r="B37" s="19" t="str">
+        <x:v>Stormspire branch. Up to five primary targets. Every fifth hit per tower and enemy adds 21 bonus damage and resets charges. Stuns for 0.4 seconds with 2-second stun immunity. Suspended storm rings and charge symbols.</x:v>
+      </x:c>
+      <x:c r="C37" s="19"/>
+      <x:c r="D37" s="19"/>
+      <x:c r="E37" s="19"/>
+      <x:c r="F37" s="19"/>
+      <x:c r="G37" s="19"/>
+    </x:row>
   </x:sheetData>
+  <x:mergeCells>
+    <x:mergeCell ref="B30:G30"/>
+    <x:mergeCell ref="B31:G31"/>
+    <x:mergeCell ref="B32:G32"/>
+    <x:mergeCell ref="B33:G33"/>
+    <x:mergeCell ref="B34:G34"/>
+    <x:mergeCell ref="B35:G35"/>
+    <x:mergeCell ref="B36:G36"/>
+    <x:mergeCell ref="B37:G37"/>
+  </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra2310f470a0f4f81"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R219f4eb4ec9f473b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -821,7 +1179,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5d614008df8741b8"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd0cad0b28fa448e4"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>